<commit_message>
Create 'vignettes/development_notes.Rmd' Other tidy-ups.
</commit_message>
<xml_diff>
--- a/vignettes/country_aggregates/aggregate_names_map.xlsx
+++ b/vignettes/country_aggregates/aggregate_names_map.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWHELDON\Documents\repos\FPCounts\FPEMglobal\vignettes\country_aggregates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A32D98-980F-43F3-947C-B2152B6D14D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F47FB81-4E37-4A74-BA69-A52925ACE421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29355" yWindow="570" windowWidth="24525" windowHeight="16560" xr2:uid="{8589771B-062C-4C93-94B3-AD3B542CB34C}"/>
+    <workbookView xWindow="3360" yWindow="756" windowWidth="27360" windowHeight="16536" xr2:uid="{8589771B-062C-4C93-94B3-AD3B542CB34C}"/>
   </bookViews>
   <sheets>
     <sheet name="aggregate_names_map" sheetId="1" r:id="rId1"/>
+    <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="105">
   <si>
     <t>parent_type</t>
   </si>
@@ -41,27 +42,9 @@
     <t>development_groups</t>
   </si>
   <si>
-    <t>Developed countries</t>
-  </si>
-  <si>
-    <t>More developed countries</t>
-  </si>
-  <si>
-    <t>Developing countries</t>
-  </si>
-  <si>
-    <t>Less developed countries</t>
-  </si>
-  <si>
-    <t>Developing (excl. China)</t>
-  </si>
-  <si>
     <t>Other developing countries</t>
   </si>
   <si>
-    <t>Less developed countries, excluding China</t>
-  </si>
-  <si>
     <t>Least developed countries</t>
   </si>
   <si>
@@ -236,9 +219,6 @@
     <t>[May 2022] Developed</t>
   </si>
   <si>
-    <t>[May 2022] Developing</t>
-  </si>
-  <si>
     <t>[SDG_regions_LLDCs_SIDS] Small island developing States (SIDS)</t>
   </si>
   <si>
@@ -357,6 +337,18 @@
   </si>
   <si>
     <t>[sdg_regions] Sub SaharanAfrica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sheet 'aggregate_names_map' contains mappings between aggregates that contain the same countries. Some of these are given different names in different aggregation schemes. </t>
+  </si>
+  <si>
+    <t>Developed countries / More developed countries</t>
+  </si>
+  <si>
+    <t>Developing countries / Less developed countries</t>
+  </si>
+  <si>
+    <t>Developing (excl. China) / Less developed countries, excluding China</t>
   </si>
 </sst>
 </file>
@@ -907,8 +899,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C4918238-F9F1-4A31-932E-3DFC2D631BBE}" name="Table2" displayName="Table2" ref="A1:F62" totalsRowShown="0">
-  <autoFilter ref="A1:F62" xr:uid="{C4918238-F9F1-4A31-932E-3DFC2D631BBE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C4918238-F9F1-4A31-932E-3DFC2D631BBE}" name="Table2" displayName="Table2" ref="A1:F56" totalsRowShown="0">
+  <autoFilter ref="A1:F56" xr:uid="{C4918238-F9F1-4A31-932E-3DFC2D631BBE}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{800B1CEE-7BA4-465A-B56C-776B92726D5B}" name="parent_type"/>
     <tableColumn id="2" xr3:uid="{155907CC-0EF9-438C-A3B8-3807FD05E443}" name="WPP 2024"/>
@@ -1238,12 +1230,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0116A2-7B2B-4CF8-8C9F-85B3BE327C9E}">
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.33203125" customWidth="1"/>
-    <col min="3" max="3" width="35.21875" customWidth="1"/>
+    <col min="2" max="2" width="68.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.109375" customWidth="1"/>
     <col min="4" max="4" width="49.5546875" customWidth="1"/>
     <col min="5" max="5" width="56.77734375" customWidth="1"/>
     <col min="6" max="6" width="25.33203125" customWidth="1"/>
@@ -1254,19 +1246,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C1" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="E1" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F1" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1274,16 +1266,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1291,16 +1283,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -1308,16 +1300,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -1325,16 +1317,16 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>3</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -1342,16 +1334,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -1359,16 +1348,10 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" t="s">
-        <v>101</v>
-      </c>
-      <c r="F7" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -1376,223 +1359,196 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
-      </c>
-      <c r="F8" t="s">
-        <v>65</v>
+        <v>95</v>
+      </c>
+      <c r="E8" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>96</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
-      </c>
-      <c r="F9" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
-      </c>
-      <c r="F10" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
-      </c>
-      <c r="F11" t="s">
-        <v>67</v>
+        <v>97</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
-        <v>97</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" t="s">
-        <v>103</v>
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
         <v>18</v>
       </c>
-      <c r="D16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" t="s">
-        <v>68</v>
-      </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
-      <c r="D17" t="s">
-        <v>104</v>
-      </c>
-      <c r="E17" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
       </c>
+      <c r="D19" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
         <v>22</v>
       </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
         <v>23</v>
       </c>
+      <c r="D21" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B22" t="s">
         <v>24</v>
       </c>
+      <c r="D22" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
       </c>
+      <c r="D23" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
         <v>26</v>
       </c>
-      <c r="C24" t="s">
-        <v>13</v>
+      <c r="D24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
       </c>
-      <c r="D25" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
         <v>28</v>
@@ -1600,10 +1556,13 @@
       <c r="D26" t="s">
         <v>28</v>
       </c>
+      <c r="E26" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
         <v>29</v>
@@ -1614,7 +1573,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
         <v>30</v>
@@ -1625,7 +1584,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
         <v>31</v>
@@ -1633,10 +1592,13 @@
       <c r="D29" t="s">
         <v>31</v>
       </c>
+      <c r="E29" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B30" t="s">
         <v>32</v>
@@ -1644,21 +1606,21 @@
       <c r="D30" t="s">
         <v>32</v>
       </c>
-      <c r="E30" t="s">
-        <v>81</v>
-      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
         <v>33</v>
       </c>
+      <c r="D31" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
         <v>34</v>
@@ -1667,12 +1629,12 @@
         <v>34</v>
       </c>
       <c r="E32" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
         <v>35</v>
@@ -1680,10 +1642,13 @@
       <c r="D33" t="s">
         <v>35</v>
       </c>
+      <c r="E33" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
         <v>36</v>
@@ -1691,24 +1656,27 @@
       <c r="D34" t="s">
         <v>36</v>
       </c>
+      <c r="E34" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
         <v>37</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
+        <v>98</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
         <v>38</v>
@@ -1719,7 +1687,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
         <v>39</v>
@@ -1730,7 +1698,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
         <v>40</v>
@@ -1739,12 +1707,12 @@
         <v>40</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
         <v>41</v>
@@ -1752,13 +1720,10 @@
       <c r="D39" t="s">
         <v>41</v>
       </c>
-      <c r="E39" t="s">
-        <v>80</v>
-      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B40" t="s">
         <v>42</v>
@@ -1766,38 +1731,35 @@
       <c r="D40" t="s">
         <v>42</v>
       </c>
-      <c r="E40" t="s">
-        <v>79</v>
-      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B41" t="s">
         <v>43</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
-      </c>
-      <c r="E41" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B42" t="s">
         <v>44</v>
       </c>
       <c r="D42" t="s">
-        <v>44</v>
+        <v>99</v>
+      </c>
+      <c r="E42" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B43" t="s">
         <v>45</v>
@@ -1805,10 +1767,13 @@
       <c r="D43" t="s">
         <v>45</v>
       </c>
+      <c r="E43" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B44" t="s">
         <v>46</v>
@@ -1816,13 +1781,10 @@
       <c r="D44" t="s">
         <v>46</v>
       </c>
-      <c r="E44" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B45" t="s">
         <v>47</v>
@@ -1833,7 +1795,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B46" t="s">
         <v>48</v>
@@ -1841,199 +1803,127 @@
       <c r="D46" t="s">
         <v>48</v>
       </c>
+      <c r="E46" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
         <v>49</v>
       </c>
-      <c r="D47" t="s">
-        <v>49</v>
+      <c r="E47" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B48" t="s">
         <v>50</v>
       </c>
-      <c r="D48" t="s">
-        <v>106</v>
-      </c>
-      <c r="E48" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
         <v>51</v>
       </c>
-      <c r="D49" t="s">
-        <v>51</v>
-      </c>
       <c r="E49" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
         <v>52</v>
       </c>
-      <c r="D50" t="s">
-        <v>52</v>
+      <c r="E50" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
         <v>53</v>
       </c>
+      <c r="C51" t="s">
+        <v>8</v>
+      </c>
       <c r="D51" t="s">
-        <v>53</v>
+        <v>100</v>
+      </c>
+      <c r="E51" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B52" t="s">
-        <v>54</v>
+        <v>53</v>
+      </c>
+      <c r="C52" t="s">
+        <v>8</v>
       </c>
       <c r="D52" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="E52" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E53" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B54" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="E54" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E55" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E56" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>17</v>
-      </c>
-      <c r="B57" t="s">
-        <v>59</v>
-      </c>
-      <c r="C57" t="s">
-        <v>14</v>
-      </c>
-      <c r="D57" t="s">
-        <v>107</v>
-      </c>
-      <c r="E57" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>17</v>
-      </c>
-      <c r="B58" t="s">
-        <v>59</v>
-      </c>
-      <c r="C58" t="s">
-        <v>14</v>
-      </c>
-      <c r="D58" t="s">
-        <v>107</v>
-      </c>
-      <c r="E58" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>17</v>
-      </c>
-      <c r="B59" t="s">
-        <v>60</v>
-      </c>
-      <c r="E59" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>17</v>
-      </c>
-      <c r="B60" t="s">
-        <v>61</v>
-      </c>
-      <c r="E60" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>17</v>
-      </c>
-      <c r="B61" t="s">
-        <v>62</v>
-      </c>
-      <c r="E61" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>17</v>
-      </c>
-      <c r="B62" t="s">
-        <v>63</v>
-      </c>
-      <c r="E62" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -2043,4 +1933,22 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00235C06-C0F0-490D-AF49-6A70FF206D47}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="111.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>